<commit_message>
Update credit score 2026-10-14 18:15:25
</commit_message>
<xml_diff>
--- a/customers/ali.xlsx
+++ b/customers/ali.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>نام طرف حساب :</t>
   </si>
@@ -73,6 +73,12 @@
   </si>
   <si>
     <t>سیگار تخم مرغ</t>
+  </si>
+  <si>
+    <t>1405/07/22</t>
+  </si>
+  <si>
+    <t>وجه</t>
   </si>
 </sst>
 </file>
@@ -590,17 +596,23 @@
     <row r="7" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
+      <c r="C7" s="10">
+        <v>1800000</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -610,7 +622,7 @@
     <row r="9" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -620,7 +632,7 @@
     <row r="10" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -630,7 +642,7 @@
     <row r="11" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -640,7 +652,7 @@
     <row r="12" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -650,7 +662,7 @@
     <row r="13" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -660,7 +672,7 @@
     <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -670,7 +682,7 @@
     <row r="15" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -680,7 +692,7 @@
     <row r="16" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -690,7 +702,7 @@
     <row r="17" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -700,7 +712,7 @@
     <row r="18" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -710,7 +722,7 @@
     <row r="19" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -720,7 +732,7 @@
     <row r="20" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
@@ -730,7 +742,7 @@
     <row r="21" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="7"/>
@@ -740,7 +752,7 @@
     <row r="22" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -750,7 +762,7 @@
     <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
         <f t="shared" si="0"/>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
@@ -765,7 +777,7 @@
       </c>
       <c r="C24" s="13">
         <f xml:space="preserve"> SUM(C3:C23)</f>
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
@@ -782,7 +794,7 @@
       <c r="B26" s="13"/>
       <c r="C26" s="14">
         <f>A23</f>
-        <v>1887000</v>
+        <v>87000</v>
       </c>
       <c r="D26" s="13" t="s">
         <v>6</v>

</xml_diff>